<commit_message>
feat: add project imports and application approval flow
</commit_message>
<xml_diff>
--- a/server/templates/import/科研项目数据标准导入模板.xlsx
+++ b/server/templates/import/科研项目数据标准导入模板.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="157">
   <si>
     <t>科研项目数据标准导入模板</t>
   </si>
@@ -40,31 +40,31 @@
     <t>导入说明和字段字典仅供查看，不作为业务数据导入。</t>
   </si>
   <si>
-    <t>project_year</t>
+    <t>项目所属年度</t>
   </si>
   <si>
-    <t>project_group</t>
+    <t>组别</t>
   </si>
   <si>
-    <t>project_code</t>
+    <t>项目编号</t>
   </si>
   <si>
-    <t>title</t>
+    <t>作品名称</t>
   </si>
   <si>
-    <t>category</t>
+    <t>项目类别</t>
   </si>
   <si>
-    <t>approval_date</t>
+    <t>立项日期</t>
   </si>
   <si>
-    <t>approval_type</t>
+    <t>立项类型</t>
   </si>
   <si>
-    <t>status</t>
+    <t>项目状态</t>
   </si>
   <si>
-    <t>remark</t>
+    <t>备注</t>
   </si>
   <si>
     <t>2026</t>
@@ -94,34 +94,37 @@
     <t>示例备注</t>
   </si>
   <si>
-    <t>person_type</t>
+    <t>人员类型</t>
   </si>
   <si>
-    <t>name</t>
+    <t>姓名</t>
   </si>
   <si>
-    <t>student_no</t>
+    <t>学号</t>
   </si>
   <si>
-    <t>teacher_no</t>
+    <t>工号</t>
   </si>
   <si>
-    <t>college</t>
+    <t>学院</t>
   </si>
   <si>
-    <t>unit</t>
+    <t>单位</t>
   </si>
   <si>
-    <t>phone</t>
+    <t>电话</t>
   </si>
   <si>
-    <t>qq</t>
+    <t>QQ</t>
   </si>
   <si>
-    <t>email</t>
+    <t>邮箱</t>
   </si>
   <si>
-    <t>account_status</t>
+    <t>职务或职称</t>
+  </si>
+  <si>
+    <t>账号状态</t>
   </si>
   <si>
     <t>student</t>
@@ -175,16 +178,16 @@
     <t>指导老师示例</t>
   </si>
   <si>
-    <t>person_identifier</t>
+    <t>人员编号</t>
   </si>
   <si>
-    <t>role</t>
+    <t>项目身份</t>
   </si>
   <si>
-    <t>is_primary_owner</t>
+    <t>是否主要负责人</t>
   </si>
   <si>
-    <t>joined_at</t>
+    <t>加入日期</t>
   </si>
   <si>
     <t>owner</t>
@@ -202,16 +205,16 @@
     <t>0</t>
   </si>
   <si>
-    <t>check_phase</t>
+    <t>检查阶段</t>
   </si>
   <si>
-    <t>research_log_count</t>
+    <t>研究日志数量</t>
   </si>
   <si>
-    <t>rating</t>
+    <t>评级</t>
   </si>
   <si>
-    <t>checked_at</t>
+    <t>检查日期</t>
   </si>
   <si>
     <t>midterm</t>
@@ -244,22 +247,22 @@
     <t>阶段检查示例</t>
   </si>
   <si>
-    <t>budget_amount</t>
+    <t>报销额度</t>
   </si>
   <si>
-    <t>midterm_claim_amount</t>
+    <t>中期申报金额</t>
   </si>
   <si>
-    <t>midterm_actual_amount</t>
+    <t>中期实际金额</t>
   </si>
   <si>
-    <t>stage_claim_amount</t>
+    <t>阶段申报金额</t>
   </si>
   <si>
-    <t>stage_actual_amount</t>
+    <t>阶段实际金额</t>
   </si>
   <si>
-    <t>remaining_amount</t>
+    <t>剩余额度</t>
   </si>
   <si>
     <t>3000.00</t>
@@ -280,106 +283,208 @@
     <t>报销示例</t>
   </si>
   <si>
-    <t>字段</t>
+    <t>字段名</t>
+  </si>
+  <si>
+    <t>模板表头</t>
   </si>
   <si>
     <t>说明</t>
   </si>
   <si>
+    <t>project_year</t>
+  </si>
+  <si>
     <t>项目所属年度；四位年份</t>
+  </si>
+  <si>
+    <t>project_group</t>
   </si>
   <si>
     <t>组别；可空</t>
   </si>
   <si>
+    <t>project_code</t>
+  </si>
+  <si>
     <t>项目编号；必填且唯一，按文本保存</t>
+  </si>
+  <si>
+    <t>title</t>
   </si>
   <si>
     <t>作品或项目名称；必填</t>
   </si>
   <si>
+    <t>category</t>
+  </si>
+  <si>
     <t>项目类别；可空</t>
+  </si>
+  <si>
+    <t>approval_date</t>
   </si>
   <si>
     <t>立项日期；YYYY-MM-DD</t>
   </si>
   <si>
+    <t>approval_type</t>
+  </si>
+  <si>
     <t>立项类型；first / supplement</t>
+  </si>
+  <si>
+    <t>status</t>
   </si>
   <si>
     <t>项目状态；draft / active / checking / completed / archived / stopped</t>
   </si>
   <si>
+    <t>person_type</t>
+  </si>
+  <si>
     <t>人员类型；student / teacher</t>
+  </si>
+  <si>
+    <t>name</t>
   </si>
   <si>
     <t>姓名；必填</t>
   </si>
   <si>
+    <t>student_no</t>
+  </si>
+  <si>
     <t>学号；学生必填且唯一，按文本保存</t>
+  </si>
+  <si>
+    <t>teacher_no</t>
   </si>
   <si>
     <t>工号；老师必填且唯一，按文本保存</t>
   </si>
   <si>
+    <t>college</t>
+  </si>
+  <si>
     <t>学院；可空</t>
+  </si>
+  <si>
+    <t>unit</t>
   </si>
   <si>
     <t>单位；可空</t>
   </si>
   <si>
+    <t>phone</t>
+  </si>
+  <si>
     <t>电话；按文本保存</t>
+  </si>
+  <si>
+    <t>qq</t>
   </si>
   <si>
     <t>QQ；按文本保存</t>
   </si>
   <si>
+    <t>email</t>
+  </si>
+  <si>
     <t>邮箱；可空</t>
+  </si>
+  <si>
+    <t>account_status</t>
   </si>
   <si>
     <t>账号状态；none / enabled / disabled</t>
   </si>
   <si>
+    <t>person_identifier</t>
+  </si>
+  <si>
     <t>人员编号；学生填学号，老师填工号，按文本保存</t>
+  </si>
+  <si>
+    <t>role</t>
   </si>
   <si>
     <t>项目身份；owner / member / advisor</t>
   </si>
   <si>
+    <t>is_primary_owner</t>
+  </si>
+  <si>
     <t>是否主要负责人；主要负责人填 1，其他填 0</t>
+  </si>
+  <si>
+    <t>joined_at</t>
   </si>
   <si>
     <t>加入日期；YYYY-MM-DD，可空</t>
   </si>
   <si>
+    <t>check_phase</t>
+  </si>
+  <si>
     <t>检查阶段；midterm / stage</t>
+  </si>
+  <si>
+    <t>research_log_count</t>
   </si>
   <si>
     <t>研究日志数量；非负整数</t>
   </si>
   <si>
+    <t>rating</t>
+  </si>
+  <si>
     <t>评级；按原始记录填写</t>
+  </si>
+  <si>
+    <t>checked_at</t>
   </si>
   <si>
     <t>检查日期；YYYY-MM-DD</t>
   </si>
   <si>
+    <t>budget_amount</t>
+  </si>
+  <si>
     <t>报销额度；数字，最多两位小数</t>
+  </si>
+  <si>
+    <t>midterm_claim_amount</t>
   </si>
   <si>
     <t>中期申报金额；数字，最多两位小数</t>
   </si>
   <si>
+    <t>midterm_actual_amount</t>
+  </si>
+  <si>
     <t>中期实际金额；数字，最多两位小数</t>
+  </si>
+  <si>
+    <t>stage_claim_amount</t>
   </si>
   <si>
     <t>阶段申报金额；数字，最多两位小数</t>
   </si>
   <si>
+    <t>stage_actual_amount</t>
+  </si>
+  <si>
     <t>阶段实际金额；数字，最多两位小数</t>
   </si>
   <si>
+    <t>remaining_amount</t>
+  </si>
+  <si>
     <t>剩余额度；数字，最多两位小数</t>
+  </si>
+  <si>
+    <t>remark</t>
   </si>
   <si>
     <t>备注；可空</t>
@@ -852,13 +957,9 @@
   <dimension ref="A1:I1000"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="20" style="4" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="7" width="21" customWidth="1"/>
-    <col min="8" max="9" width="14" customWidth="1"/>
+    <col min="1" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="14" style="4" customWidth="1"/>
+    <col min="4" max="9" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -10925,15 +11026,11 @@
   <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="4" width="18" style="4" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="1" max="2" width="14" customWidth="1"/>
+    <col min="3" max="4" width="14" style="4" customWidth="1"/>
+    <col min="5" max="6" width="14" customWidth="1"/>
     <col min="7" max="8" width="14" style="4" customWidth="1"/>
-    <col min="9" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="22" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
+    <col min="9" max="12" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -10965,10 +11062,10 @@
         <v>33</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L1" s="6" t="s">
         <v>15</v>
@@ -10976,78 +11073,78 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>38</v>
+      <c r="G2" s="8" t="s">
+        <v>41</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="H2" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="H2" s="8" t="s">
-        <v>41</v>
+      <c r="G3" s="8" t="s">
+        <v>48</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="H3" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="G3" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="H3" s="8" t="s">
-        <v>38</v>
-      </c>
       <c r="I3" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -24037,13 +24134,12 @@
   <dimension ref="A1:G1000"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="20" style="4" customWidth="1"/>
-    <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="25" style="4" customWidth="1"/>
+    <col min="1" max="1" width="14" style="4" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="14" style="4" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="17" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -24054,16 +24150,16 @@
         <v>25</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>15</v>
@@ -24074,22 +24170,22 @@
         <v>18</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>21</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -24097,22 +24193,22 @@
         <v>18</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>21</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -31126,12 +31222,8 @@
   <dimension ref="A1:F1000"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="20" style="4" customWidth="1"/>
-    <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="1" max="1" width="14" style="4" customWidth="1"/>
+    <col min="2" max="6" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -31139,16 +31231,16 @@
         <v>9</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F1" s="6" t="s">
         <v>15</v>
@@ -31159,19 +31251,19 @@
         <v>18</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -31179,19 +31271,19 @@
         <v>18</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -35202,14 +35294,8 @@
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="20" style="4" customWidth="1"/>
-    <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="29" customWidth="1"/>
-    <col min="5" max="5" width="26" customWidth="1"/>
-    <col min="6" max="6" width="27" customWidth="1"/>
-    <col min="7" max="7" width="24" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="1" max="1" width="14" style="4" customWidth="1"/>
+    <col min="2" max="8" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -35217,22 +35303,22 @@
         <v>9</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H1" s="6" t="s">
         <v>15</v>
@@ -35243,25 +35329,25 @@
         <v>18</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>82</v>
-      </c>
       <c r="H2" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -35273,283 +35359,386 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="72" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="72" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" s="6" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>89</v>
+      <c r="C2" s="3" t="s">
+        <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>90</v>
+      <c r="C3" s="3" t="s">
+        <v>94</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>91</v>
+      <c r="C4" s="3" t="s">
+        <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>92</v>
+      <c r="C5" s="3" t="s">
+        <v>98</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>93</v>
+      <c r="C6" s="3" t="s">
+        <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>94</v>
+      <c r="C7" s="3" t="s">
+        <v>102</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>95</v>
+      <c r="C8" s="3" t="s">
+        <v>104</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>96</v>
+      <c r="C9" s="3" t="s">
+        <v>106</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>97</v>
+      <c r="C10" s="3" t="s">
+        <v>108</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>98</v>
+      <c r="C11" s="3" t="s">
+        <v>110</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>99</v>
+      <c r="C12" s="3" t="s">
+        <v>112</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>100</v>
+      <c r="C13" s="3" t="s">
+        <v>114</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>101</v>
+      <c r="C14" s="3" t="s">
+        <v>116</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>102</v>
+      <c r="C15" s="3" t="s">
+        <v>118</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="3" t="s">
-        <v>103</v>
+      <c r="C16" s="3" t="s">
+        <v>120</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>104</v>
+      <c r="C17" s="3" t="s">
+        <v>122</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>105</v>
+      <c r="C18" s="3" t="s">
+        <v>124</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>34</v>
+        <v>125</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>106</v>
+        <v>35</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C19" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>52</v>
+        <v>127</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
         <v>53</v>
       </c>
+      <c r="C20" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="B21" s="3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
         <v>54</v>
       </c>
+      <c r="C21" s="3" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="B22" s="3" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
         <v>55</v>
       </c>
+      <c r="C22" s="3" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>133</v>
+      </c>
       <c r="B23" s="3" t="s">
-        <v>110</v>
+        <v>56</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C23" s="3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>61</v>
+        <v>135</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
         <v>62</v>
       </c>
+      <c r="C24" s="3" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>137</v>
+      </c>
       <c r="B25" s="3" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
         <v>63</v>
       </c>
+      <c r="C25" s="3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>139</v>
+      </c>
       <c r="B26" s="3" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
         <v>64</v>
       </c>
+      <c r="C26" s="3" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="B27" s="3" t="s">
-        <v>114</v>
+        <v>65</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C27" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>75</v>
+        <v>143</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
         <v>76</v>
       </c>
+      <c r="C28" s="3" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>145</v>
+      </c>
       <c r="B29" s="3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
         <v>77</v>
       </c>
+      <c r="C29" s="3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>147</v>
+      </c>
       <c r="B30" s="3" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
         <v>78</v>
       </c>
+      <c r="C30" s="3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>149</v>
+      </c>
       <c r="B31" s="3" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
         <v>79</v>
       </c>
+      <c r="C31" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>151</v>
+      </c>
       <c r="B32" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
         <v>80</v>
       </c>
+      <c r="C32" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="B33" s="3" t="s">
-        <v>120</v>
+        <v>81</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C33" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B34" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B34" s="3" t="s">
-        <v>121</v>
+      <c r="C34" s="3" t="s">
+        <v>156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>